<commit_message>
Name the three levels in the forms
The forms asked for a level of 1, 2 or 3 without saying what any of
them meant. Each level now carries a short name in the dropdowns, the
helper text, the reference sheet and the matching markdown rows.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -2807,7 +2807,7 @@
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -2985,7 +2985,7 @@
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>1, 2 or 3, from your Platform Control Levels.</t>
+          <t>Level 1 Hand-scoped, Level 2 Classification ceiling, Level 3 Policy as code. Defined in your Platform Control Levels.</t>
         </is>
       </c>
       <c r="B17" s="32" t="n"/>
@@ -3814,7 +3814,7 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C16 C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Level 1,Level 2,Level 3"</formula1>
+      <formula1>"Level 1 — Hand-scoped,Level 2 — Classification ceiling,Level 3 — Policy as code"</formula1>
     </dataValidation>
     <dataValidation sqref="F78:F87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
@@ -3844,7 +3844,7 @@
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -3950,7 +3950,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Monitoring level of the platform it runs on: 1, 2 or 3</t>
+          <t>Monitoring level of the platform it runs on: Level 1 Tool call log, Level 2 Run records, Level 3 Replay and test</t>
         </is>
       </c>
       <c r="B11" s="15" t="n"/>
@@ -5089,7 +5089,7 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C10 C11 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Level 1,Level 2,Level 3"</formula1>
+      <formula1>"Level 1 — Tool call log,Level 2 — Run records,Level 3 — Replay and test"</formula1>
     </dataValidation>
     <dataValidation sqref="B18:B25 E47:E54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Partly"</formula1>
@@ -6319,7 +6319,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="86" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -6560,7 +6560,7 @@
       <c r="A24" s="32" t="n"/>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Level 1 — Hand-scoped</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -6573,7 +6573,7 @@
       <c r="A25" s="32" t="n"/>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 2 — Classification ceiling</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
@@ -6586,7 +6586,7 @@
       <c r="A26" s="32" t="n"/>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 3 — Policy as code</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
@@ -6619,7 +6619,7 @@
       <c r="A29" s="32" t="n"/>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Level 1 — Tool call log</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -6632,7 +6632,7 @@
       <c r="A30" s="32" t="n"/>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 2 — Run records</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
@@ -6645,7 +6645,7 @@
       <c r="A31" s="32" t="n"/>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 3 — Replay and test</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Say who answers the regulation question
Question 3 left it open whether the agent's team could decide which
regulations reach the process. Name the adviser in the question itself,
in the standard, in the design document and in the forms.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Agent Design" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Classification" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2a Floor Anchors" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Platform &amp; Sign-off" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Monitoring" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Audit &amp; Assurance" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Reference" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="1 Agent Design" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2 Classification" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2a Floor Anchors" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="3 Platform &amp; Sign-off" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="4 Monitoring" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="5 Audit &amp; Assurance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="6 Reference" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'1 Agent Design'!$1:$2</definedName>
@@ -230,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -336,6 +336,10 @@
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -410,39 +414,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1714500" cy="771525"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -972,7 +943,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2171,7 +2141,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Which regulations reach this process? Name them, or write "none that we have identified" and say who looked.</t>
+          <t>Which regulations reach this process? Name them, or write "none that we have identified". Either way, name the legal, compliance or privacy adviser who determined it.</t>
         </is>
       </c>
       <c r="C13" s="35" t="n"/>
@@ -2249,8 +2219,12 @@
       <c r="E18" s="35" t="n"/>
       <c r="F18" s="34" t="n"/>
     </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="32" t="n"/>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>Question 3 is not a question this form answers, and not one the agent’s team answers on its own. Which regulations reach a process is a determination from whoever advises your company on regulation — legal, compliance, or privacy. Record their answer in the row and name them; "none that we have identified" with nobody named behind it leaves the row unanswered.</t>
+        </is>
+      </c>
       <c r="B19" s="32" t="n"/>
       <c r="C19" s="32" t="n"/>
       <c r="D19" s="32" t="n"/>
@@ -2385,7 +2359,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="31">
+  <mergeCells count="32">
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A27:F27"/>
@@ -2407,6 +2381,7 @@
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="E15:F15"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="A32:B32"/>

</xml_diff>

<commit_message>
Patch the workbook in place instead of rewriting it
The previous commit round-tripped the file through openpyxl, which
dropped the cover image. Same two edits, applied to the sheet XML.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1 Agent Design" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2 Classification" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2a Floor Anchors" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="3 Platform &amp; Sign-off" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="4 Monitoring" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="5 Audit &amp; Assurance" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="6 Reference" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Agent Design" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Classification" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2a Floor Anchors" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Platform &amp; Sign-off" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Monitoring" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Audit &amp; Assurance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Reference" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'1 Agent Design'!$1:$2</definedName>
@@ -230,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -336,10 +336,6 @@
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1" indent="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,6 +410,39 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="771525"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -943,6 +972,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2219,8 +2249,8 @@
       <c r="E18" s="35" t="n"/>
       <c r="F18" s="34" t="n"/>
     </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="39" t="inlineStr">
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Question 3 is not a question this form answers, and not one the agent’s team answers on its own. Which regulations reach a process is a determination from whoever advises your company on regulation — legal, compliance, or privacy. Record their answer in the row and name them; "none that we have identified" with nobody named behind it leaves the row unanswered.</t>
         </is>
@@ -2360,6 +2390,7 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="32">
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A27:F27"/>
@@ -2381,7 +2412,6 @@
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="E15:F15"/>
-    <mergeCell ref="A19:F19"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="A32:B32"/>

</xml_diff>

<commit_message>
Say which way the money goes in question 4
"Moves money" was reading as spending. Name the three kinds - out, in,
and committed - in the question, the anchors, the value ceiling and the
forms, and say that value which is not currency counts.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -1494,10 +1494,10 @@
       <c r="F48" s="36" t="n"/>
       <c r="G48" s="34" t="n"/>
     </row>
-    <row r="49" ht="13" customHeight="1">
+    <row r="49" ht="70" customHeight="70">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>The most money or value the agent can move in one action, and in one day. Write "none" if there is no ceiling, and expect the Classification sheet to charge you for it.</t>
+          <t>The most money or value the agent can move in one action, and in one day, stated for each kind of movement it can make: money out (payments, refunds, credits, discounts), money in (charges, invoices, collections), and commitments that become money later (orders, contracts, billable provisioning). Value that is not currency counts: inventory, store credit, points, gift cards, licences. Write "none" against a kind that has no ceiling, and expect the Classification sheet to charge you for it.</t>
         </is>
       </c>
     </row>
@@ -2179,13 +2179,13 @@
       <c r="E13" s="35" t="n"/>
       <c r="F13" s="34" t="n"/>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14" ht="48" customHeight="48">
       <c r="A14" s="17" t="n">
         <v>4</v>
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>How much money or value can it move, in one action and in one day?</t>
+          <t>How much money or value can it move, in one action and in one day? Answer for each kind of movement it can make: money out, money in, and commitments that become money later.</t>
         </is>
       </c>
       <c r="C14" s="35" t="n"/>
@@ -2627,22 +2627,22 @@
       </c>
       <c r="C11" s="35" t="inlineStr">
         <is>
-          <t>It moves no money or value.</t>
+          <t>It moves no money or value: none out, none in, and it commits none.</t>
         </is>
       </c>
       <c r="D11" s="35" t="inlineStr">
         <is>
-          <t>It moves money or value within a ceiling that covers both one action and one day, recorded in its design document.</t>
+          <t>Every kind of movement it makes is within a ceiling that covers both one action and one day, recorded in its design document.</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>The ceiling covers one action but not one day, or nothing approves the actions that reach it.</t>
+          <t>A ceiling covers one action but not one day, or nothing approves the actions that reach it.</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>No ceiling, or a ceiling the agent observes itself rather than one the platform enforces.</t>
+          <t>A kind of movement it can make has no ceiling, or has one the agent observes itself rather than one the platform enforces.</t>
         </is>
       </c>
     </row>
@@ -2774,10 +2774,10 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="44" customHeight="1">
+    <row r="17" ht="100" customHeight="100">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Question 4 sets no amount, and this pack names none. What a given agent may move is the value ceiling in section 3 of its Agent Design sheet, accepted by whoever signs it off. The anchors judge the shape of the control instead: whether a ceiling exists, whether it covers a day as well as an action, and whether the platform enforces it or the agent is trusted to observe it. Question 7 is the one row where the anchors describe supervision instead of damage: it is what turns the other seven into risk.</t>
+          <t>Question 4 covers three kinds of movement, and most agents that reach it do more than one: money out (paying, refunding, crediting, discounting), money in (charging, invoicing, collecting) and commitments that become money later (orders, contracts, billable provisioning). Value that is not currency counts on the same footing: inventory, store credit, points, gift cards, licences. Answer for every kind the agent can do, name a ceiling for each, and take the highest floor any of them sets. Question 4 sets no amount, and this pack names none. What a given agent may move is the value ceiling in section 3 of its Agent Design sheet, accepted by whoever signs it off. The anchors judge the shape of the control instead: whether a ceiling exists, whether it covers a day as well as an action, and whether the platform enforces it or the agent is trusted to observe it. Question 7 is the one row where the anchors describe supervision instead of damage: it is what turns the other seven into risk.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Start the other clocks somewhere
Four claims whose start, end or threshold was unstated: what continuous
means for the access check, what credential lifetime does to revocation,
how you find out a run did not happen, and when the reversal window opens.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -2199,7 +2199,7 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Can you undo what it does? Name the action that is hardest to undo, and how long you have.</t>
+          <t>Can you undo what it does? Name the action that is hardest to undo, and how long you have from the moment it takes effect.</t>
         </is>
       </c>
       <c r="C15" s="35" t="n"/>
@@ -2664,12 +2664,12 @@
       </c>
       <c r="D12" s="35" t="inlineStr">
         <is>
-          <t>Reversible by the team within one working day.</t>
+          <t>Reversible by the team within one working day of the action taking effect.</t>
         </is>
       </c>
       <c r="E12" s="35" t="inlineStr">
         <is>
-          <t>Reversible only with another party's help, or beyond one working day.</t>
+          <t>Reversible only with another party's help, or beyond one working day of the action taking effect.</t>
         </is>
       </c>
       <c r="F12" s="35" t="inlineStr">
@@ -4278,7 +4278,7 @@
     <row r="40" ht="56" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>How you would know they had stopped running</t>
+          <t>How you would know they had stopped running, and how long after the run that did not happen</t>
         </is>
       </c>
       <c r="B40" s="15" t="n"/>
@@ -5641,7 +5641,7 @@
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>How you would know the evals had stopped running</t>
+          <t>How you would know the evals had stopped running, and how long after the run that did not happen</t>
         </is>
       </c>
       <c r="B49" s="15" t="n"/>

</xml_diff>

<commit_message>
Record what holds each grant, row by row
The form asked where the grant list is enforced once, for the whole
agent, and had three rows to transcribe it into. Give the table a
per-row enforcement column, twelve rows, and constrained answers; add
the mirror of the over-grant row for limits nothing can enforce; and say
in the ladder that Level 3 needs a grant list code can read.

The sheet was also protected against inserting rows, so a thirty-grant
agent could not be recorded at all. Inserting and deleting rows is now
allowed there.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -2807,7 +2807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3158,7 +3158,11 @@
           <t>Wider, narrower, or the same</t>
         </is>
       </c>
-      <c r="E33" s="16" t="n"/>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Where it is enforced</t>
+        </is>
+      </c>
       <c r="F33" s="15" t="n"/>
     </row>
     <row r="34" ht="26" customHeight="1">
@@ -3166,7 +3170,7 @@
       <c r="B34" s="35" t="n"/>
       <c r="C34" s="34" t="n"/>
       <c r="D34" s="35" t="n"/>
-      <c r="E34" s="36" t="n"/>
+      <c r="E34" s="35" t="n"/>
       <c r="F34" s="34" t="n"/>
     </row>
     <row r="35" ht="26" customHeight="1">
@@ -3174,7 +3178,7 @@
       <c r="B35" s="35" t="n"/>
       <c r="C35" s="34" t="n"/>
       <c r="D35" s="35" t="n"/>
-      <c r="E35" s="36" t="n"/>
+      <c r="E35" s="35" t="n"/>
       <c r="F35" s="34" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
@@ -3182,117 +3186,100 @@
       <c r="B36" s="35" t="n"/>
       <c r="C36" s="34" t="n"/>
       <c r="D36" s="35" t="n"/>
-      <c r="E36" s="36" t="n"/>
+      <c r="E36" s="35" t="n"/>
       <c r="F36" s="34" t="n"/>
     </row>
     <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="32" t="n"/>
-      <c r="B37" s="32" t="n"/>
-      <c r="C37" s="32" t="n"/>
-      <c r="D37" s="32" t="n"/>
-      <c r="E37" s="32" t="n"/>
-      <c r="F37" s="32" t="n"/>
-    </row>
-    <row r="38" ht="56" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
+      <c r="A37" s="35" t="n"/>
+      <c r="B37" s="35" t="n"/>
+      <c r="C37" s="34" t="n"/>
+      <c r="D37" s="35" t="n"/>
+      <c r="E37" s="35" t="n"/>
+      <c r="F37" s="34" t="n"/>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="35" t="n"/>
+      <c r="B38" s="35" t="n"/>
+      <c r="C38" s="34" t="n"/>
+      <c r="D38" s="35" t="n"/>
+      <c r="E38" s="35" t="n"/>
+      <c r="F38" s="34" t="n"/>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="A39" s="35" t="n"/>
+      <c r="B39" s="35" t="n"/>
+      <c r="C39" s="34" t="n"/>
+      <c r="D39" s="35" t="n"/>
+      <c r="E39" s="35" t="n"/>
+      <c r="F39" s="34" t="n"/>
+    </row>
+    <row r="40" ht="26" customHeight="1">
+      <c r="A40" s="35" t="n"/>
+      <c r="B40" s="35" t="n"/>
+      <c r="C40" s="34" t="n"/>
+      <c r="D40" s="35" t="n"/>
+      <c r="E40" s="35" t="n"/>
+      <c r="F40" s="34" t="n"/>
+    </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="35" t="n"/>
+      <c r="B41" s="35" t="n"/>
+      <c r="C41" s="34" t="n"/>
+      <c r="D41" s="35" t="n"/>
+      <c r="E41" s="35" t="n"/>
+      <c r="F41" s="34" t="n"/>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="35" t="n"/>
+      <c r="B42" s="35" t="n"/>
+      <c r="C42" s="34" t="n"/>
+      <c r="D42" s="35" t="n"/>
+      <c r="E42" s="35" t="n"/>
+      <c r="F42" s="34" t="n"/>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="35" t="n"/>
+      <c r="B43" s="35" t="n"/>
+      <c r="C43" s="34" t="n"/>
+      <c r="D43" s="35" t="n"/>
+      <c r="E43" s="35" t="n"/>
+      <c r="F43" s="34" t="n"/>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="35" t="n"/>
+      <c r="B44" s="35" t="n"/>
+      <c r="C44" s="34" t="n"/>
+      <c r="D44" s="35" t="n"/>
+      <c r="E44" s="35" t="n"/>
+      <c r="F44" s="34" t="n"/>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="35" t="n"/>
+      <c r="B45" s="35" t="n"/>
+      <c r="C45" s="34" t="n"/>
+      <c r="D45" s="35" t="n"/>
+      <c r="E45" s="35" t="n"/>
+      <c r="F45" s="34" t="n"/>
+    </row>
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>Add rows until every row of section 3 has one here — select a row inside the table and insert, then copy an existing row down so the dropdowns come with it. A summary of thirty grants is not this table. "Nowhere" in the last column is an honest answer: the row is a sentence in a document rather than a control, and it belongs in section C as remaining risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="32" t="n"/>
+      <c r="B47" s="32" t="n"/>
+      <c r="C47" s="32" t="n"/>
+      <c r="D47" s="32" t="n"/>
+      <c r="E47" s="32" t="n"/>
+      <c r="F47" s="32" t="n"/>
+    </row>
+    <row r="48" ht="56" customHeight="1">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>Anything narrower than the design document asks for</t>
-        </is>
-      </c>
-      <c r="B38" s="15" t="n"/>
-      <c r="C38" s="35" t="n"/>
-      <c r="D38" s="36" t="n"/>
-      <c r="E38" s="36" t="n"/>
-      <c r="F38" s="34" t="n"/>
-    </row>
-    <row r="39" ht="13" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
-        <is>
-          <t>Say what the agent cannot do as a result, and whether anybody has worked around it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="56" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>What is granted that the design document does not list</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="n"/>
-      <c r="C40" s="35" t="n"/>
-      <c r="D40" s="36" t="n"/>
-      <c r="E40" s="36" t="n"/>
-      <c r="F40" s="34" t="n"/>
-    </row>
-    <row r="41" ht="27" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>Anything the agent can reach that section 3 does not name. This should be empty. Where it is not, carry it into section C as remaining risk. Do not fix it quietly and leave this blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="32" t="n"/>
-      <c r="B42" s="32" t="n"/>
-      <c r="C42" s="32" t="n"/>
-      <c r="D42" s="32" t="n"/>
-      <c r="E42" s="32" t="n"/>
-      <c r="F42" s="32" t="n"/>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
-        <is>
-          <t>B.  What the evals found   (against the setup in section A, not a development configuration)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>Which evals you ran</t>
-        </is>
-      </c>
-      <c r="B44" s="15" t="n"/>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="36" t="n"/>
-      <c r="E44" s="36" t="n"/>
-      <c r="F44" s="34" t="n"/>
-    </row>
-    <row r="45" ht="56" customHeight="1">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>Adversarial testing performed, and what it was tested against</t>
-        </is>
-      </c>
-      <c r="B45" s="15" t="n"/>
-      <c r="C45" s="35" t="n"/>
-      <c r="D45" s="36" t="n"/>
-      <c r="E45" s="36" t="n"/>
-      <c r="F45" s="34" t="n"/>
-    </row>
-    <row r="46" ht="26" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>For any agent that reads content it did not author, whether it can be talked into something is what the sign-off most needs to know. Name what you tested against from OWASP's Top 10 for Agentic Applications, the same list the Monitoring sheet's playbook works from.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>Against which configuration, matching section A</t>
-        </is>
-      </c>
-      <c r="B47" s="15" t="n"/>
-      <c r="C47" s="35" t="n"/>
-      <c r="D47" s="36" t="n"/>
-      <c r="E47" s="36" t="n"/>
-      <c r="F47" s="34" t="n"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="10" t="inlineStr">
-        <is>
-          <t>Date of the run</t>
         </is>
       </c>
       <c r="B48" s="15" t="n"/>
@@ -3301,41 +3288,36 @@
       <c r="E48" s="36" t="n"/>
       <c r="F48" s="34" t="n"/>
     </row>
-    <row r="49" ht="56" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>What they found</t>
-        </is>
-      </c>
-      <c r="B49" s="15" t="n"/>
-      <c r="C49" s="35" t="n"/>
-      <c r="D49" s="36" t="n"/>
-      <c r="E49" s="36" t="n"/>
-      <c r="F49" s="34" t="n"/>
-    </row>
-    <row r="50" ht="13" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>This is what the person signing off is accepting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="10" t="inlineStr">
-        <is>
-          <t>What you changed because of it</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="n"/>
-      <c r="C51" s="35" t="n"/>
-      <c r="D51" s="36" t="n"/>
-      <c r="E51" s="36" t="n"/>
-      <c r="F51" s="34" t="n"/>
+    <row r="49" ht="13" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>Say what the agent cannot do as a result, and whether anybody has worked around it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="56" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>What is granted that the design document does not list</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="n"/>
+      <c r="C50" s="35" t="n"/>
+      <c r="D50" s="36" t="n"/>
+      <c r="E50" s="36" t="n"/>
+      <c r="F50" s="34" t="n"/>
+    </row>
+    <row r="51" ht="27" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>Anything the agent can reach that section 3 does not name. This should be empty. Where it is not, carry it into section C as remaining risk. Do not fix it quietly and leave this blank.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="56" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>What you know you did NOT test</t>
+          <t>Limits the platform cannot express</t>
         </is>
       </c>
       <c r="B52" s="15" t="n"/>
@@ -3344,44 +3326,44 @@
       <c r="E52" s="36" t="n"/>
       <c r="F52" s="34" t="n"/>
     </row>
-    <row r="53" ht="13" customHeight="1">
+    <row r="53" ht="40" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>This is where stage 4 monitoring has to begin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="10" t="inlineStr">
-        <is>
-          <t>Where the results are kept</t>
-        </is>
-      </c>
-      <c r="B54" s="15" t="n"/>
-      <c r="C54" s="35" t="n"/>
-      <c r="D54" s="36" t="n"/>
-      <c r="E54" s="36" t="n"/>
-      <c r="F54" s="34" t="n"/>
-    </row>
-    <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="32" t="n"/>
-      <c r="B55" s="32" t="n"/>
-      <c r="C55" s="32" t="n"/>
-      <c r="D55" s="32" t="n"/>
-      <c r="E55" s="32" t="n"/>
-      <c r="F55" s="32" t="n"/>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>C.  Sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
+          <t>Every row of section 3 whose granularity is "not enforceable here": a boundary declared in stage 1 that nothing here can hold. Say what the agent can reach as a result, and carry these into section C as remaining risk. The row above is access nobody meant to grant; this one is a limit nobody can enforce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="26" customHeight="1">
+      <c r="A54" s="32" t="n"/>
+      <c r="B54" s="32" t="n"/>
+      <c r="C54" s="32" t="n"/>
+      <c r="D54" s="32" t="n"/>
+      <c r="E54" s="32" t="n"/>
+      <c r="F54" s="32" t="n"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>B.  What the evals found   (against the setup in section A, not a development configuration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>Which evals you ran</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="n"/>
+      <c r="C56" s="35" t="n"/>
+      <c r="D56" s="36" t="n"/>
+      <c r="E56" s="36" t="n"/>
+      <c r="F56" s="34" t="n"/>
+    </row>
+    <row r="57" ht="56" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Adversarial testing performed, and what it was tested against</t>
         </is>
       </c>
       <c r="B57" s="15" t="n"/>
@@ -3390,22 +3372,17 @@
       <c r="E57" s="36" t="n"/>
       <c r="F57" s="34" t="n"/>
     </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="10" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="B58" s="15" t="n"/>
-      <c r="C58" s="35" t="n"/>
-      <c r="D58" s="36" t="n"/>
-      <c r="E58" s="36" t="n"/>
-      <c r="F58" s="34" t="n"/>
+    <row r="58" ht="26" customHeight="1">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>For any agent that reads content it did not author, whether it can be talked into something is what the sign-off most needs to know. Name what you tested against from OWASP's Top 10 for Agentic Applications, the same list the Monitoring sheet's playbook works from.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Against which configuration, matching section A</t>
         </is>
       </c>
       <c r="B59" s="15" t="n"/>
@@ -3417,7 +3394,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>Version of the design document signed</t>
+          <t>Date of the run</t>
         </is>
       </c>
       <c r="B60" s="15" t="n"/>
@@ -3426,10 +3403,10 @@
       <c r="E60" s="36" t="n"/>
       <c r="F60" s="34" t="n"/>
     </row>
-    <row r="61" ht="30" customHeight="1">
+    <row r="61" ht="56" customHeight="1">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>Version of this record signed</t>
+          <t>What they found</t>
         </is>
       </c>
       <c r="B61" s="15" t="n"/>
@@ -3438,22 +3415,17 @@
       <c r="E61" s="36" t="n"/>
       <c r="F61" s="34" t="n"/>
     </row>
-    <row r="62" ht="56" customHeight="1">
-      <c r="A62" s="10" t="inlineStr">
-        <is>
-          <t>The risk that is left, stated in their words</t>
-        </is>
-      </c>
-      <c r="B62" s="15" t="n"/>
-      <c r="C62" s="35" t="n"/>
-      <c r="D62" s="36" t="n"/>
-      <c r="E62" s="36" t="n"/>
-      <c r="F62" s="34" t="n"/>
+    <row r="62" ht="13" customHeight="1">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>This is what the person signing off is accepting.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>Any classification floor lowered by a compensating control</t>
+          <t>What you changed because of it</t>
         </is>
       </c>
       <c r="B63" s="15" t="n"/>
@@ -3462,60 +3434,56 @@
       <c r="E63" s="36" t="n"/>
       <c r="F63" s="34" t="n"/>
     </row>
-    <row r="64" ht="13" customHeight="1">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>A floor lowered in the design document and not repeated here has not been accepted by anybody.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="56" customHeight="1">
-      <c r="A65" s="10" t="inlineStr">
-        <is>
-          <t>Conditions on the sign-off, and when it must be looked at again</t>
-        </is>
-      </c>
-      <c r="B65" s="15" t="n"/>
-      <c r="C65" s="35" t="n"/>
-      <c r="D65" s="36" t="n"/>
-      <c r="E65" s="36" t="n"/>
-      <c r="F65" s="34" t="n"/>
+    <row r="64" ht="56" customHeight="1">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t>What you know you did NOT test</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="n"/>
+      <c r="C64" s="35" t="n"/>
+      <c r="D64" s="36" t="n"/>
+      <c r="E64" s="36" t="n"/>
+      <c r="F64" s="34" t="n"/>
+    </row>
+    <row r="65" ht="13" customHeight="1">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>This is where stage 4 monitoring has to begin.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="30" customHeight="1">
-      <c r="A66" s="24" t="inlineStr">
-        <is>
-          <t>THE LEVEL GAP.  The agent's classification names a platform control level and a monitoring level that an agent in it requires. Where the level applied is lower, the gap is accepted here, by name, or it is not accepted at all.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="10" t="inlineStr">
-        <is>
-          <t>Platform control level the classification requires, and the level applied</t>
-        </is>
-      </c>
-      <c r="B67" s="15" t="n"/>
-      <c r="C67" s="35" t="n"/>
-      <c r="D67" s="36" t="n"/>
-      <c r="E67" s="36" t="n"/>
-      <c r="F67" s="34" t="n"/>
-    </row>
-    <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="10" t="inlineStr">
-        <is>
-          <t>Monitoring level the classification requires, and the level applied</t>
-        </is>
-      </c>
-      <c r="B68" s="15" t="n"/>
-      <c r="C68" s="35" t="n"/>
-      <c r="D68" s="36" t="n"/>
-      <c r="E68" s="36" t="n"/>
-      <c r="F68" s="34" t="n"/>
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>Where the results are kept</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="n"/>
+      <c r="C66" s="35" t="n"/>
+      <c r="D66" s="36" t="n"/>
+      <c r="E66" s="36" t="n"/>
+      <c r="F66" s="34" t="n"/>
+    </row>
+    <row r="67" ht="26" customHeight="1">
+      <c r="A67" s="32" t="n"/>
+      <c r="B67" s="32" t="n"/>
+      <c r="C67" s="32" t="n"/>
+      <c r="D67" s="32" t="n"/>
+      <c r="E67" s="32" t="n"/>
+      <c r="F67" s="32" t="n"/>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>C.  Sign-off</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>Who accepts the gap, by name</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B69" s="15" t="n"/>
@@ -3527,7 +3495,7 @@
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="10" t="inlineStr">
         <is>
-          <t>The date by which it closes</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="B70" s="15" t="n"/>
@@ -3539,7 +3507,7 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>How many consecutive sign-offs have accepted this same gap</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B71" s="15" t="n"/>
@@ -3548,280 +3516,442 @@
       <c r="E71" s="36" t="n"/>
       <c r="F71" s="34" t="n"/>
     </row>
-    <row r="72" ht="26" customHeight="1">
-      <c r="A72" s="13" t="inlineStr">
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>Version of the design document signed</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="n"/>
+      <c r="C72" s="35" t="n"/>
+      <c r="D72" s="36" t="n"/>
+      <c r="E72" s="36" t="n"/>
+      <c r="F72" s="34" t="n"/>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Version of this record signed</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="n"/>
+      <c r="C73" s="35" t="n"/>
+      <c r="D73" s="36" t="n"/>
+      <c r="E73" s="36" t="n"/>
+      <c r="F73" s="34" t="n"/>
+    </row>
+    <row r="74" ht="56" customHeight="1">
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t>The risk that is left, stated in their words</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="n"/>
+      <c r="C74" s="35" t="n"/>
+      <c r="D74" s="36" t="n"/>
+      <c r="E74" s="36" t="n"/>
+      <c r="F74" s="34" t="n"/>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>Any classification floor lowered by a compensating control</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="n"/>
+      <c r="C75" s="35" t="n"/>
+      <c r="D75" s="36" t="n"/>
+      <c r="E75" s="36" t="n"/>
+      <c r="F75" s="34" t="n"/>
+    </row>
+    <row r="76" ht="13" customHeight="1">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>A floor lowered in the design document and not repeated here has not been accepted by anybody.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="56" customHeight="1">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>Conditions on the sign-off, and when it must be looked at again</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="n"/>
+      <c r="C77" s="35" t="n"/>
+      <c r="D77" s="36" t="n"/>
+      <c r="E77" s="36" t="n"/>
+      <c r="F77" s="34" t="n"/>
+    </row>
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="24" t="inlineStr">
+        <is>
+          <t>THE LEVEL GAP.  The agent's classification names a platform control level and a monitoring level that an agent in it requires. Where the level applied is lower, the gap is accepted here, by name, or it is not accepted at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>Platform control level the classification requires, and the level applied</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="n"/>
+      <c r="C79" s="35" t="n"/>
+      <c r="D79" s="36" t="n"/>
+      <c r="E79" s="36" t="n"/>
+      <c r="F79" s="34" t="n"/>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>Monitoring level the classification requires, and the level applied</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="n"/>
+      <c r="C80" s="35" t="n"/>
+      <c r="D80" s="36" t="n"/>
+      <c r="E80" s="36" t="n"/>
+      <c r="F80" s="34" t="n"/>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>Who accepts the gap, by name</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="n"/>
+      <c r="C81" s="35" t="n"/>
+      <c r="D81" s="36" t="n"/>
+      <c r="E81" s="36" t="n"/>
+      <c r="F81" s="34" t="n"/>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>The date by which it closes</t>
+        </is>
+      </c>
+      <c r="B82" s="15" t="n"/>
+      <c r="C82" s="35" t="n"/>
+      <c r="D82" s="36" t="n"/>
+      <c r="E82" s="36" t="n"/>
+      <c r="F82" s="34" t="n"/>
+    </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>How many consecutive sign-offs have accepted this same gap</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="n"/>
+      <c r="C83" s="35" t="n"/>
+      <c r="D83" s="36" t="n"/>
+      <c r="E83" s="36" t="n"/>
+      <c r="F83" s="34" t="n"/>
+    </row>
+    <row r="84" ht="26" customHeight="1">
+      <c r="A84" s="13" t="inlineStr">
         <is>
           <t>Answer the last row honestly. A gap accepted once is a legitimate decision made under time pressure. A gap accepted three times in a row is a decision nobody is making, and this count is the only thing on any of these forms that would show it.</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="26" customHeight="1">
-      <c r="A73" s="32" t="n"/>
-      <c r="B73" s="32" t="n"/>
-      <c r="C73" s="32" t="n"/>
-      <c r="D73" s="32" t="n"/>
-      <c r="E73" s="32" t="n"/>
-      <c r="F73" s="32" t="n"/>
-    </row>
-    <row r="74" ht="26" customHeight="1">
-      <c r="A74" s="24" t="inlineStr">
+    <row r="85" ht="26" customHeight="1">
+      <c r="A85" s="32" t="n"/>
+      <c r="B85" s="32" t="n"/>
+      <c r="C85" s="32" t="n"/>
+      <c r="D85" s="32" t="n"/>
+      <c r="E85" s="32" t="n"/>
+      <c r="F85" s="32" t="n"/>
+    </row>
+    <row r="86" ht="26" customHeight="1">
+      <c r="A86" s="24" t="inlineStr">
         <is>
           <t>The sign-off is against the two versions named above. When live behavior stops matching the description it was granted against, it is void until somebody looks again.</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="32" t="n"/>
-      <c r="B75" s="32" t="n"/>
-      <c r="C75" s="32" t="n"/>
-      <c r="D75" s="32" t="n"/>
-      <c r="E75" s="32" t="n"/>
-      <c r="F75" s="32" t="n"/>
-    </row>
-    <row r="76" ht="22" customHeight="1">
-      <c r="A76" s="9" t="inlineStr">
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="32" t="n"/>
+      <c r="B87" s="32" t="n"/>
+      <c r="C87" s="32" t="n"/>
+      <c r="D87" s="32" t="n"/>
+      <c r="E87" s="32" t="n"/>
+      <c r="F87" s="32" t="n"/>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
         <is>
           <t>D.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="28" customHeight="1">
-      <c r="A77" s="14" t="inlineStr">
+    <row r="89" ht="28" customHeight="1">
+      <c r="A89" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B77" s="14" t="inlineStr">
+      <c r="B89" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C77" s="14" t="inlineStr">
+      <c r="C89" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D77" s="14" t="inlineStr">
+      <c r="D89" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E77" s="14" t="inlineStr">
+      <c r="E89" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F77" s="14" t="inlineStr">
+      <c r="F89" s="14" t="inlineStr">
         <is>
           <t>Did it need a new sign-off</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="26" customHeight="1">
-      <c r="A78" s="35" t="n"/>
-      <c r="B78" s="35" t="n"/>
-      <c r="C78" s="35" t="n"/>
-      <c r="D78" s="35" t="n"/>
-      <c r="E78" s="35" t="n"/>
-      <c r="F78" s="35" t="n"/>
-    </row>
-    <row r="79" ht="26" customHeight="1">
-      <c r="A79" s="35" t="n"/>
-      <c r="B79" s="35" t="n"/>
-      <c r="C79" s="35" t="n"/>
-      <c r="D79" s="35" t="n"/>
-      <c r="E79" s="35" t="n"/>
-      <c r="F79" s="35" t="n"/>
-    </row>
-    <row r="80" ht="26" customHeight="1">
-      <c r="A80" s="35" t="n"/>
-      <c r="B80" s="35" t="n"/>
-      <c r="C80" s="35" t="n"/>
-      <c r="D80" s="35" t="n"/>
-      <c r="E80" s="35" t="n"/>
-      <c r="F80" s="35" t="n"/>
-    </row>
-    <row r="81" ht="26" customHeight="1">
-      <c r="A81" s="35" t="n"/>
-      <c r="B81" s="35" t="n"/>
-      <c r="C81" s="35" t="n"/>
-      <c r="D81" s="35" t="n"/>
-      <c r="E81" s="35" t="n"/>
-      <c r="F81" s="35" t="n"/>
-    </row>
-    <row r="82" ht="26" customHeight="1">
-      <c r="A82" s="35" t="n"/>
-      <c r="B82" s="35" t="n"/>
-      <c r="C82" s="35" t="n"/>
-      <c r="D82" s="35" t="n"/>
-      <c r="E82" s="35" t="n"/>
-      <c r="F82" s="35" t="n"/>
-    </row>
-    <row r="83" ht="26" customHeight="1">
-      <c r="A83" s="35" t="n"/>
-      <c r="B83" s="35" t="n"/>
-      <c r="C83" s="35" t="n"/>
-      <c r="D83" s="35" t="n"/>
-      <c r="E83" s="35" t="n"/>
-      <c r="F83" s="35" t="n"/>
-    </row>
-    <row r="84" ht="26" customHeight="1">
-      <c r="A84" s="35" t="n"/>
-      <c r="B84" s="35" t="n"/>
-      <c r="C84" s="35" t="n"/>
-      <c r="D84" s="35" t="n"/>
-      <c r="E84" s="35" t="n"/>
-      <c r="F84" s="35" t="n"/>
-    </row>
-    <row r="85" ht="26" customHeight="1">
-      <c r="A85" s="35" t="n"/>
-      <c r="B85" s="35" t="n"/>
-      <c r="C85" s="35" t="n"/>
-      <c r="D85" s="35" t="n"/>
-      <c r="E85" s="35" t="n"/>
-      <c r="F85" s="35" t="n"/>
-    </row>
-    <row r="86" ht="26" customHeight="1">
-      <c r="A86" s="35" t="n"/>
-      <c r="B86" s="35" t="n"/>
-      <c r="C86" s="35" t="n"/>
-      <c r="D86" s="35" t="n"/>
-      <c r="E86" s="35" t="n"/>
-      <c r="F86" s="35" t="n"/>
-    </row>
-    <row r="87" ht="26" customHeight="1">
-      <c r="A87" s="35" t="n"/>
-      <c r="B87" s="35" t="n"/>
-      <c r="C87" s="35" t="n"/>
-      <c r="D87" s="35" t="n"/>
-      <c r="E87" s="35" t="n"/>
-      <c r="F87" s="35" t="n"/>
-    </row>
-    <row r="88" ht="26" customHeight="1">
-      <c r="A88" s="13" t="inlineStr">
+    <row r="90" ht="26" customHeight="1">
+      <c r="A90" s="35" t="n"/>
+      <c r="B90" s="35" t="n"/>
+      <c r="C90" s="35" t="n"/>
+      <c r="D90" s="35" t="n"/>
+      <c r="E90" s="35" t="n"/>
+      <c r="F90" s="35" t="n"/>
+    </row>
+    <row r="91" ht="26" customHeight="1">
+      <c r="A91" s="35" t="n"/>
+      <c r="B91" s="35" t="n"/>
+      <c r="C91" s="35" t="n"/>
+      <c r="D91" s="35" t="n"/>
+      <c r="E91" s="35" t="n"/>
+      <c r="F91" s="35" t="n"/>
+    </row>
+    <row r="92" ht="26" customHeight="1">
+      <c r="A92" s="35" t="n"/>
+      <c r="B92" s="35" t="n"/>
+      <c r="C92" s="35" t="n"/>
+      <c r="D92" s="35" t="n"/>
+      <c r="E92" s="35" t="n"/>
+      <c r="F92" s="35" t="n"/>
+    </row>
+    <row r="93" ht="26" customHeight="1">
+      <c r="A93" s="35" t="n"/>
+      <c r="B93" s="35" t="n"/>
+      <c r="C93" s="35" t="n"/>
+      <c r="D93" s="35" t="n"/>
+      <c r="E93" s="35" t="n"/>
+      <c r="F93" s="35" t="n"/>
+    </row>
+    <row r="94" ht="26" customHeight="1">
+      <c r="A94" s="35" t="n"/>
+      <c r="B94" s="35" t="n"/>
+      <c r="C94" s="35" t="n"/>
+      <c r="D94" s="35" t="n"/>
+      <c r="E94" s="35" t="n"/>
+      <c r="F94" s="35" t="n"/>
+    </row>
+    <row r="95" ht="26" customHeight="1">
+      <c r="A95" s="35" t="n"/>
+      <c r="B95" s="35" t="n"/>
+      <c r="C95" s="35" t="n"/>
+      <c r="D95" s="35" t="n"/>
+      <c r="E95" s="35" t="n"/>
+      <c r="F95" s="35" t="n"/>
+    </row>
+    <row r="96" ht="26" customHeight="1">
+      <c r="A96" s="35" t="n"/>
+      <c r="B96" s="35" t="n"/>
+      <c r="C96" s="35" t="n"/>
+      <c r="D96" s="35" t="n"/>
+      <c r="E96" s="35" t="n"/>
+      <c r="F96" s="35" t="n"/>
+    </row>
+    <row r="97" ht="26" customHeight="1">
+      <c r="A97" s="35" t="n"/>
+      <c r="B97" s="35" t="n"/>
+      <c r="C97" s="35" t="n"/>
+      <c r="D97" s="35" t="n"/>
+      <c r="E97" s="35" t="n"/>
+      <c r="F97" s="35" t="n"/>
+    </row>
+    <row r="98" ht="26" customHeight="1">
+      <c r="A98" s="35" t="n"/>
+      <c r="B98" s="35" t="n"/>
+      <c r="C98" s="35" t="n"/>
+      <c r="D98" s="35" t="n"/>
+      <c r="E98" s="35" t="n"/>
+      <c r="F98" s="35" t="n"/>
+    </row>
+    <row r="99" ht="26" customHeight="1">
+      <c r="A99" s="35" t="n"/>
+      <c r="B99" s="35" t="n"/>
+      <c r="C99" s="35" t="n"/>
+      <c r="D99" s="35" t="n"/>
+      <c r="E99" s="35" t="n"/>
+      <c r="F99" s="35" t="n"/>
+    </row>
+    <row r="100" ht="26" customHeight="1">
+      <c r="A100" s="13" t="inlineStr">
         <is>
           <t>A model version bump, a framework upgrade, a new tool, or a change of host all produce a row. Answer the last column every time, because an auditor will ask which changes went live without a fresh sign-off.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="109">
-    <mergeCell ref="C52:F52"/>
-    <mergeCell ref="C61:F61"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <mergeCells count="131">
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A66:F66"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="C56:F56"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C77:F77"/>
+    <mergeCell ref="C71:F71"/>
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A70:B70"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C80:F80"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="C73:F73"/>
+    <mergeCell ref="C59:F59"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C57:F57"/>
+    <mergeCell ref="A83:B83"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="A80:B80"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="C66:F66"/>
+    <mergeCell ref="C11:F11"/>
     <mergeCell ref="C13:F13"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="C62:F62"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C75:F75"/>
+    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="C54:F54"/>
-    <mergeCell ref="C63:F63"/>
     <mergeCell ref="C10:F10"/>
-    <mergeCell ref="A64:F64"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A62:B62"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C67:F67"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="C69:F69"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C40:F40"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A63:B63"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A88:F88"/>
-    <mergeCell ref="C71:F71"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A74:F74"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="C57:F57"/>
-    <mergeCell ref="A69:B69"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="A76:F76"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="C68:F68"/>
+    <mergeCell ref="C60:F60"/>
+    <mergeCell ref="C64:F64"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C79:F79"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C83:F83"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A62:F62"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A82:B82"/>
+    <mergeCell ref="C69:F69"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="C74:F74"/>
+    <mergeCell ref="C70:F70"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A86:F86"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="A100:F100"/>
+    <mergeCell ref="A78:F78"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="A88:F88"/>
+    <mergeCell ref="A79:B79"/>
+    <mergeCell ref="C81:F81"/>
+    <mergeCell ref="A65:F65"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="C63:F63"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C72:F72"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C61:F61"/>
+    <mergeCell ref="C82:F82"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="C52:F52"/>
     <mergeCell ref="A53:F53"/>
-    <mergeCell ref="C58:F58"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D35:F35"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C65:F65"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C47:F47"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="C44:F44"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="C51:F51"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="C60:F60"/>
-    <mergeCell ref="C70:F70"/>
-    <mergeCell ref="C48:F48"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="C38:F38"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C49:F49"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C59:F59"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="A58:B58"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="4">
+    <dataValidation sqref="D34:D45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Wider,Narrower,The same"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E34:E45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Gateway,Policy engine,Scoped credential,Tool wrapper,Nowhere"</formula1>
+    </dataValidation>
     <dataValidation sqref="C16 C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Level 1 — Hand-scoped,Level 2 — Classification ceiling,Level 3 — Policy as code"</formula1>
     </dataValidation>
-    <dataValidation sqref="F78:F87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F90:F99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Let every sheet grow
Row insertion was blocked on all eight sheets, so every table was capped
at the rows it shipped with.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -961,7 +961,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
@@ -1878,7 +1878,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="103">
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A73:B73"/>
@@ -2388,7 +2388,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="32">
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="E12:F12"/>
@@ -2789,7 +2789,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="5">
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
@@ -5103,7 +5103,7 @@
       <c r="F99" s="34" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="116">
     <mergeCell ref="C39:F39"/>
     <mergeCell ref="E62:F62"/>
@@ -6294,7 +6294,7 @@
       <c r="F103" s="34" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="120">
     <mergeCell ref="A64:B64"/>
     <mergeCell ref="E62:F62"/>
@@ -6983,7 +6983,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="8">
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
Let every sheet grow, the other way round
The previous commit set insertRows and deleteRows to 1 on all eight
sheets, which locks both. In sheetProtection a 1 means the action is
locked, not permitted, and openpyxl exposes the raw attribute under a
name that reads the other way. The workbook shipped with both at 0 and
tells people to insert rows into the grant list, so they go back to 0.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -928,7 +928,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
@@ -1851,7 +1851,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="104">
     <mergeCell ref="C68:G68"/>
     <mergeCell ref="A17:G17"/>
@@ -2357,7 +2357,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="32">
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="A24:B24"/>
@@ -2758,7 +2758,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="5">
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
@@ -3852,7 +3852,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="143">
     <mergeCell ref="C52:F52"/>
     <mergeCell ref="C61:F61"/>
@@ -3895,8 +3895,8 @@
     <mergeCell ref="A51:F51"/>
     <mergeCell ref="A60:F60"/>
     <mergeCell ref="A68:B68"/>
+    <mergeCell ref="C27:F27"/>
     <mergeCell ref="B41:C41"/>
-    <mergeCell ref="C27:F27"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="A30:B30"/>
@@ -5205,7 +5205,7 @@
       <c r="F103" s="34" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="113">
     <mergeCell ref="C39:F39"/>
     <mergeCell ref="E62:F62"/>
@@ -6393,7 +6393,7 @@
       <c r="F103" s="34" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="120">
     <mergeCell ref="A64:B64"/>
     <mergeCell ref="E62:F62"/>
@@ -7082,7 +7082,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="8">
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
Stop calling the working copy a release
The stamp on every sheet, form and note said September 2026 Draft, which
is the last thing released, not what is in here. Say working copy, and
tell a reader to cite a release, because this one changes under them.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -748,7 +748,7 @@
       <c r="A8" s="32" t="n"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>September 2026 Draft</t>
+          <t>Unreleased working copy</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, September 2026 Draft&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, Unreleased working copy&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -970,7 +970,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>September 2026 Draft</t>
+          <t>Unreleased working copy</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -1976,7 +1976,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, September 2026 Draft&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, Unreleased working copy&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2012,7 +2012,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>September 2026 Draft</t>
+          <t>Unreleased working copy</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -2401,7 +2401,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, September 2026 Draft&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, Unreleased working copy&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2437,7 +2437,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>September 2026 Draft</t>
+          <t>Unreleased working copy</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>September 2026 Draft</t>
+          <t>Unreleased working copy</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -4019,7 +4019,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, September 2026 Draft&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, Unreleased working copy&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -4055,7 +4055,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>September 2026 Draft</t>
+          <t>Unreleased working copy</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -5333,7 +5333,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, September 2026 Draft&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, Unreleased working copy&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5369,7 +5369,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>September 2026 Draft</t>
+          <t>Unreleased working copy</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -6534,7 +6534,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, September 2026 Draft&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, Unreleased working copy&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6567,7 +6567,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>September 2026 Draft</t>
+          <t>Unreleased working copy</t>
         </is>
       </c>
       <c r="B2" s="32" t="n"/>
@@ -7097,7 +7097,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, September 2026 Draft&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8 &amp;K595959MACH Alliance — Agent Governance and Assurance Framework, Unreleased working copy&amp;R&amp;8 &amp;K595959&amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>